<commit_message>
Agregado apellido a la consola y reporte para flujos ATC
</commit_message>
<xml_diff>
--- a/data/maestro.xlsx
+++ b/data/maestro.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://everisgroup-my.sharepoint.com/personal/dnarvaec_emeal_nttdata_com1/Documents/Documents/Proyectos AUTO/Avianca/Automatizacion/auto_avianca/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{48F3D4DC-C1BA-440D-80D9-C9B78812467E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04CE6BB7-2B78-484A-8639-5AC6898117AC}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="8_{48F3D4DC-C1BA-440D-80D9-C9B78812467E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6EAD875A-E348-4245-A5AE-F050ECC6A449}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="2370" windowHeight="560" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="686" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="229">
   <si>
     <t>TC</t>
   </si>
@@ -642,13 +642,97 @@
   </si>
   <si>
     <t>Test 21</t>
+  </si>
+  <si>
+    <t>Tipo Flujo</t>
+  </si>
+  <si>
+    <t>Trayectos A Cambiar</t>
+  </si>
+  <si>
+    <t>Vuelo Ida Nuevo</t>
+  </si>
+  <si>
+    <t>Vuelo Vuelta Nuevo</t>
+  </si>
+  <si>
+    <t>Tarifa Nueva</t>
+  </si>
+  <si>
+    <t>Total Esperado</t>
+  </si>
+  <si>
+    <t>Requiere Pago</t>
+  </si>
+  <si>
+    <t>Medio De Pago</t>
+  </si>
+  <si>
+    <t>Resultado_Esperado</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>ATC-01</t>
+  </si>
+  <si>
+    <t>Pre condición</t>
+  </si>
+  <si>
+    <t>Cambio con pago</t>
+  </si>
+  <si>
+    <t>Ida y vuelta</t>
+  </si>
+  <si>
+    <t>Primer vuelo disponible</t>
+  </si>
+  <si>
+    <t>Primera tarifa disponible</t>
+  </si>
+  <si>
+    <t>Mayor a 0</t>
+  </si>
+  <si>
+    <t>Tarjeta de prueba</t>
+  </si>
+  <si>
+    <t>Tu reserva está confirmada</t>
+  </si>
+  <si>
+    <t>Pendiente</t>
+  </si>
+  <si>
+    <t>ATC-02</t>
+  </si>
+  <si>
+    <t>Ida</t>
+  </si>
+  <si>
+    <t>Confirmado</t>
+  </si>
+  <si>
+    <t>ATC-03</t>
+  </si>
+  <si>
+    <t>Cambio sin pago o saldo a favor</t>
+  </si>
+  <si>
+    <t>Vuelo con tarifa 0 o menor</t>
+  </si>
+  <si>
+    <t>0 o saldo a favor</t>
+  </si>
+  <si>
+    <t>Tu cambio fue realizado con éxito</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -689,16 +773,43 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -721,12 +832,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -752,6 +900,24 @@
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3752,9 +3918,189 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99263EF0-1BE3-4964-9B9B-BA2465D40400}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="5" max="5" width="17.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>202</v>
+      </c>
+      <c r="G1" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="H1" s="14" t="s">
+        <v>204</v>
+      </c>
+      <c r="I1" s="14" t="s">
+        <v>205</v>
+      </c>
+      <c r="J1" s="14" t="s">
+        <v>206</v>
+      </c>
+      <c r="K1" s="14" t="s">
+        <v>207</v>
+      </c>
+      <c r="L1" s="14" t="s">
+        <v>208</v>
+      </c>
+      <c r="M1" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="N1" s="14" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A2" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="H2" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="I2" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="J2" s="18" t="s">
+        <v>217</v>
+      </c>
+      <c r="K2" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="L2" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="M2" s="18" t="s">
+        <v>219</v>
+      </c>
+      <c r="N2" s="18" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A3" s="16" t="s">
+        <v>221</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>222</v>
+      </c>
+      <c r="G3" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="H3" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="J3" s="18" t="s">
+        <v>217</v>
+      </c>
+      <c r="K3" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="L3" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="M3" s="18" t="s">
+        <v>219</v>
+      </c>
+      <c r="N3" s="18" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A4" s="16" t="s">
+        <v>224</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>225</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="G4" s="18" t="s">
+        <v>226</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>226</v>
+      </c>
+      <c r="I4" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="J4" s="18" t="s">
+        <v>227</v>
+      </c>
+      <c r="K4" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="L4" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="M4" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="N4" s="18" t="s">
+        <v>223</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Se agregan parametrizables de vuelos de ida y vuelta
</commit_message>
<xml_diff>
--- a/data/maestro.xlsx
+++ b/data/maestro.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://everisgroup-my.sharepoint.com/personal/dnarvaec_emeal_nttdata_com1/Documents/Documents/Proyectos AUTO/Avianca/Automatizacion/auto_avianca/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="8_{48F3D4DC-C1BA-440D-80D9-C9B78812467E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6EAD875A-E348-4245-A5AE-F050ECC6A449}"/>
+  <xr:revisionPtr revIDLastSave="73" documentId="8_{48F3D4DC-C1BA-440D-80D9-C9B78812467E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96EB83F1-F7E9-4C2C-BC7E-032FCFA188C2}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="2370" windowHeight="560" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NBF_OW" sheetId="5" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="243">
   <si>
     <t>TC</t>
   </si>
@@ -726,6 +726,48 @@
   </si>
   <si>
     <t>Tu cambio fue realizado con éxito</t>
+  </si>
+  <si>
+    <t>Origen</t>
+  </si>
+  <si>
+    <t>Destino</t>
+  </si>
+  <si>
+    <t>BOG</t>
+  </si>
+  <si>
+    <t>JFK</t>
+  </si>
+  <si>
+    <t>DEN</t>
+  </si>
+  <si>
+    <t>ACA</t>
+  </si>
+  <si>
+    <t>MAD</t>
+  </si>
+  <si>
+    <t>IAD</t>
+  </si>
+  <si>
+    <t>MEX</t>
+  </si>
+  <si>
+    <t>BCN</t>
+  </si>
+  <si>
+    <t>AEP</t>
+  </si>
+  <si>
+    <t>OPO</t>
+  </si>
+  <si>
+    <t>CLO</t>
+  </si>
+  <si>
+    <t>MDE</t>
   </si>
 </sst>
 </file>
@@ -795,7 +837,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -806,6 +848,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -874,7 +922,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -919,6 +967,22 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1223,144 +1287,151 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17F2B12E-54CA-4F16-A6A7-4F29CA9834E4}">
-  <dimension ref="A1:X11"/>
+  <dimension ref="A1:Z11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.6328125" customWidth="1"/>
+    <col min="2" max="3" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>177</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="3">
+      <c r="E2" s="3">
         <v>46327</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="2">
+      <c r="I2" s="2">
         <v>1</v>
-      </c>
-      <c r="H2" s="2">
-        <v>0</v>
-      </c>
-      <c r="I2" s="2">
-        <v>0</v>
       </c>
       <c r="J2" s="2">
         <v>0</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="2">
+        <v>0</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="O2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P2" s="2" t="s">
+      <c r="Q2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="S2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="T2" s="2" t="s">
         <v>31</v>
       </c>
@@ -1374,33 +1445,39 @@
         <v>31</v>
       </c>
       <c r="X2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z2" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>178</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C3" s="3">
+      <c r="E3" s="3">
         <v>46327</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="G3" s="2">
-        <v>1</v>
-      </c>
-      <c r="H3" s="2">
-        <v>0</v>
       </c>
       <c r="I3" s="2">
         <v>1</v>
@@ -1408,38 +1485,38 @@
       <c r="J3" s="2">
         <v>0</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="2">
+        <v>1</v>
+      </c>
+      <c r="L3" s="2">
+        <v>0</v>
+      </c>
+      <c r="M3" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="N3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="O3" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="P3" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="O3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P3" s="2" t="s">
+      <c r="Q3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R3" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="Q3" s="4" t="s">
+      <c r="S3" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="T3" s="2" t="s">
         <v>31</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="V3" s="2" t="s">
         <v>31</v>
@@ -1448,141 +1525,153 @@
         <v>31</v>
       </c>
       <c r="X3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z3" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>179</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C4" s="3">
+      <c r="E4" s="3">
         <v>46327</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G4" s="2">
+      <c r="I4" s="2">
         <v>2</v>
-      </c>
-      <c r="H4" s="2">
-        <v>1</v>
-      </c>
-      <c r="I4" s="2">
-        <v>1</v>
       </c>
       <c r="J4" s="2">
         <v>1</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="K4" s="2">
+        <v>1</v>
+      </c>
+      <c r="L4" s="2">
+        <v>1</v>
+      </c>
+      <c r="M4" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="O4" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="P4" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="O4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P4" s="2" t="s">
+      <c r="Q4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R4" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="Q4" s="4" t="s">
+      <c r="S4" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="S4" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="T4" s="2" t="s">
         <v>31</v>
       </c>
       <c r="U4" s="2" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="V4" s="2" t="s">
         <v>31</v>
       </c>
       <c r="W4" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="X4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z4" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>180</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="3">
+      <c r="E5" s="3">
         <v>46327</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="G5" s="2">
+      <c r="I5" s="2">
         <v>3</v>
-      </c>
-      <c r="H5" s="2">
-        <v>2</v>
-      </c>
-      <c r="I5" s="2">
-        <v>2</v>
       </c>
       <c r="J5" s="2">
         <v>2</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="K5" s="2">
+        <v>2</v>
+      </c>
+      <c r="L5" s="2">
+        <v>2</v>
+      </c>
+      <c r="M5" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="N5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="O5" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="P5" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="O5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P5" s="2" t="s">
+      <c r="Q5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R5" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="Q5" s="4" t="s">
+      <c r="S5" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="S5" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="T5" s="2" t="s">
         <v>31</v>
       </c>
@@ -1593,70 +1682,76 @@
         <v>31</v>
       </c>
       <c r="W5" s="2" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="X5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z5" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>181</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C6" s="3">
+      <c r="E6" s="3">
         <v>46327</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="2">
+      <c r="I6" s="2">
         <v>2</v>
       </c>
-      <c r="H6" s="2">
+      <c r="J6" s="2">
         <v>1</v>
       </c>
-      <c r="I6" s="2">
+      <c r="K6" s="2">
         <v>0</v>
       </c>
-      <c r="J6" s="2">
+      <c r="L6" s="2">
         <v>0</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="M6" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="N6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M6" s="2" t="s">
+      <c r="O6" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="N6" s="2" t="s">
+      <c r="P6" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="O6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P6" s="2" t="s">
+      <c r="Q6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R6" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="Q6" s="4" t="s">
+      <c r="S6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R6" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S6" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="T6" s="2" t="s">
         <v>42</v>
       </c>
@@ -1664,261 +1759,285 @@
         <v>31</v>
       </c>
       <c r="V6" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="W6" s="2" t="s">
         <v>31</v>
       </c>
       <c r="X6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z6" s="2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>182</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C7" s="3">
+      <c r="E7" s="3">
         <v>46327</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G7" s="2">
+      <c r="I7" s="2">
         <v>2</v>
       </c>
-      <c r="H7" s="2">
+      <c r="J7" s="2">
         <v>0</v>
       </c>
-      <c r="I7" s="2">
+      <c r="K7" s="2">
         <v>1</v>
       </c>
-      <c r="J7" s="2">
+      <c r="L7" s="2">
         <v>1</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="M7" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="N7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="O7" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="P7" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="O7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P7" s="2" t="s">
+      <c r="Q7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R7" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="Q7" s="4" t="s">
+      <c r="S7" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R7" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S7" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="T7" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="U7" s="2" t="s">
         <v>31</v>
       </c>
       <c r="V7" s="2" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="W7" s="2" t="s">
         <v>31</v>
       </c>
       <c r="X7" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z7" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>183</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="3">
+      <c r="E8" s="3">
         <v>46327</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="F8" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G8" s="2">
+      <c r="I8" s="2">
         <v>5</v>
       </c>
-      <c r="H8" s="2">
+      <c r="J8" s="2">
         <v>2</v>
       </c>
-      <c r="I8" s="2">
+      <c r="K8" s="2">
         <v>1</v>
       </c>
-      <c r="J8" s="2">
+      <c r="L8" s="2">
         <v>1</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="M8" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="N8" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="O8" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="N8" s="2" t="s">
+      <c r="P8" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="O8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="P8" s="2" t="s">
+      <c r="Q8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="R8" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="Q8" s="4" t="s">
+      <c r="S8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R8" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="S8" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="T8" s="2" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="U8" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="V8" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="W8" s="2" t="s">
         <v>31</v>
       </c>
       <c r="X8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z8" s="2" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>184</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="3">
+      <c r="E9" s="3">
         <v>46327</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G9" s="2">
+      <c r="I9" s="2">
         <v>4</v>
-      </c>
-      <c r="H9" s="2">
-        <v>1</v>
-      </c>
-      <c r="I9" s="2">
-        <v>2</v>
       </c>
       <c r="J9" s="2">
         <v>1</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="K9" s="2">
+        <v>2</v>
+      </c>
+      <c r="L9" s="2">
+        <v>1</v>
+      </c>
+      <c r="M9" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="N9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M9" s="2" t="s">
+      <c r="O9" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="N9" s="2" t="s">
+      <c r="P9" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="O9" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="P9" s="2" t="s">
+      <c r="Q9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="R9" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="Q9" s="4" t="s">
+      <c r="S9" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="S9" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="T9" s="2" t="s">
         <v>31</v>
       </c>
       <c r="U9" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="V9" s="2" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="W9" s="2" t="s">
         <v>31</v>
       </c>
       <c r="X9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z9" s="2" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>185</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C10" s="3">
+      <c r="E10" s="3">
         <v>46327</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="G10" s="2">
-        <v>2</v>
-      </c>
-      <c r="H10" s="2">
-        <v>2</v>
       </c>
       <c r="I10" s="2">
         <v>2</v>
@@ -1926,33 +2045,33 @@
       <c r="J10" s="2">
         <v>2</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="K10" s="2">
+        <v>2</v>
+      </c>
+      <c r="L10" s="2">
+        <v>2</v>
+      </c>
+      <c r="M10" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="N10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M10" s="2" t="s">
+      <c r="O10" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="N10" s="2" t="s">
+      <c r="P10" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="O10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="P10" s="2" t="s">
+      <c r="Q10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="R10" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="Q10" s="4" t="s">
+      <c r="S10" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S10" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="T10" s="2" t="s">
         <v>42</v>
       </c>
@@ -1966,72 +2085,78 @@
         <v>42</v>
       </c>
       <c r="X10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z10" s="2" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>186</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="3">
+      <c r="E11" s="3">
         <v>46327</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="F11" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="G11" s="2">
+      <c r="I11" s="2">
         <v>1</v>
       </c>
-      <c r="H11" s="2">
+      <c r="J11" s="2">
         <v>3</v>
       </c>
-      <c r="I11" s="2">
+      <c r="K11" s="2">
         <v>3</v>
       </c>
-      <c r="J11" s="2">
+      <c r="L11" s="2">
         <v>2</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="M11" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="L11" s="2" t="s">
+      <c r="N11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M11" s="2" t="s">
+      <c r="O11" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="N11" s="2" t="s">
+      <c r="P11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="O11" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="P11" s="2" t="s">
+      <c r="Q11" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="R11" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="Q11" s="4" t="s">
+      <c r="S11" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R11" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S11" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="T11" s="2" t="s">
         <v>42</v>
       </c>
       <c r="U11" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="V11" s="2" t="s">
         <v>42</v>
@@ -2040,22 +2165,28 @@
         <v>31</v>
       </c>
       <c r="X11" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z11" s="2" t="s">
         <v>120</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="Q2" r:id="rId1" xr:uid="{1ADA4FCF-2D29-457F-B58C-D28286E272BE}"/>
-    <hyperlink ref="Q3" r:id="rId2" xr:uid="{83DC9D79-DA6B-4E5C-BE1C-93726DED7F58}"/>
-    <hyperlink ref="Q4" r:id="rId3" xr:uid="{B9759FFC-A172-43FE-B0DD-061AF57929D8}"/>
-    <hyperlink ref="Q5" r:id="rId4" xr:uid="{92B507E3-D79E-460C-A86F-10D6FB03A13E}"/>
-    <hyperlink ref="Q6" r:id="rId5" xr:uid="{8D80A4B4-5BAD-475E-8A25-39EF4A9029A2}"/>
-    <hyperlink ref="Q7" r:id="rId6" xr:uid="{09F21089-7AA3-400C-8735-354193A66854}"/>
-    <hyperlink ref="Q8" r:id="rId7" xr:uid="{B2FB9EEF-C3C6-4632-ACFF-9F49330DE3B5}"/>
-    <hyperlink ref="Q9" r:id="rId8" xr:uid="{61304899-7FF9-44F9-A4D5-5BBCFEFB4AF0}"/>
-    <hyperlink ref="Q10" r:id="rId9" xr:uid="{9ACACC9B-A24D-4A56-9A79-FD25E220C09C}"/>
-    <hyperlink ref="Q11" r:id="rId10" xr:uid="{F53B76E0-CE9C-4062-8AC0-CDA1FD53D1A0}"/>
+    <hyperlink ref="S2" r:id="rId1" xr:uid="{1ADA4FCF-2D29-457F-B58C-D28286E272BE}"/>
+    <hyperlink ref="S3" r:id="rId2" xr:uid="{83DC9D79-DA6B-4E5C-BE1C-93726DED7F58}"/>
+    <hyperlink ref="S4" r:id="rId3" xr:uid="{B9759FFC-A172-43FE-B0DD-061AF57929D8}"/>
+    <hyperlink ref="S5" r:id="rId4" xr:uid="{92B507E3-D79E-460C-A86F-10D6FB03A13E}"/>
+    <hyperlink ref="S6" r:id="rId5" xr:uid="{8D80A4B4-5BAD-475E-8A25-39EF4A9029A2}"/>
+    <hyperlink ref="S7" r:id="rId6" xr:uid="{09F21089-7AA3-400C-8735-354193A66854}"/>
+    <hyperlink ref="S8" r:id="rId7" xr:uid="{B2FB9EEF-C3C6-4632-ACFF-9F49330DE3B5}"/>
+    <hyperlink ref="S9" r:id="rId8" xr:uid="{61304899-7FF9-44F9-A4D5-5BBCFEFB4AF0}"/>
+    <hyperlink ref="S10" r:id="rId9" xr:uid="{9ACACC9B-A24D-4A56-9A79-FD25E220C09C}"/>
+    <hyperlink ref="S11" r:id="rId10" xr:uid="{F53B76E0-CE9C-4062-8AC0-CDA1FD53D1A0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2063,160 +2194,167 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X31"/>
+  <dimension ref="A1:Z31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.90625" customWidth="1"/>
-    <col min="3" max="3" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="7.26953125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.7265625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="17.7265625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="14" customWidth="1"/>
+    <col min="5" max="5" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.26953125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="14" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="17.7265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>187</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="5">
+      <c r="E2" s="5">
         <v>46327</v>
       </c>
-      <c r="D2" s="3">
+      <c r="F2" s="3">
         <v>46346</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="2">
+      <c r="I2" s="2">
         <v>1</v>
-      </c>
-      <c r="H2" s="2">
-        <v>0</v>
-      </c>
-      <c r="I2" s="2">
-        <v>0</v>
       </c>
       <c r="J2" s="2">
         <v>0</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="2">
+        <v>0</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="O2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P2" s="2" t="s">
+      <c r="Q2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="S2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="T2" s="2" t="s">
         <v>31</v>
       </c>
@@ -2230,215 +2368,233 @@
         <v>31</v>
       </c>
       <c r="X2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z2" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:26" s="23" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="19" t="s">
         <v>188</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="19" t="s">
+        <v>242</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>233</v>
+      </c>
+      <c r="D3" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="3">
+      <c r="E3" s="21">
         <v>46327</v>
       </c>
-      <c r="D3" s="3">
+      <c r="F3" s="21">
         <v>46346</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="G3" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="2">
+      <c r="I3" s="19">
         <v>1</v>
       </c>
-      <c r="H3" s="2">
+      <c r="J3" s="19">
         <v>1</v>
       </c>
-      <c r="I3" s="2">
+      <c r="K3" s="19">
         <v>0</v>
       </c>
-      <c r="J3" s="2">
+      <c r="L3" s="19">
         <v>0</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="M3" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="N3" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="O3" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="P3" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="O3" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="P3" s="2" t="s">
+      <c r="Q3" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="R3" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="Q3" s="4" t="s">
+      <c r="S3" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="R3" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="U3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="V3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="W3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="X3" s="2" t="s">
+      <c r="T3" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="U3" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="V3" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="W3" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="X3" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y3" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z3" s="19" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>189</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C4" s="5">
+      <c r="E4" s="5">
         <v>46327</v>
       </c>
-      <c r="D4" s="3">
+      <c r="F4" s="3">
         <v>46346</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="G4" s="2">
+      <c r="I4" s="2">
         <v>1</v>
       </c>
-      <c r="H4" s="2">
+      <c r="J4" s="2">
         <v>0</v>
       </c>
-      <c r="I4" s="2">
+      <c r="K4" s="2">
         <v>0</v>
       </c>
-      <c r="J4" s="2">
+      <c r="L4" s="2">
         <v>1</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="M4" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="O4" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="P4" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="O4" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="P4" s="2" t="s">
+      <c r="Q4" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="R4" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="Q4" s="4" t="s">
+      <c r="S4" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="S4" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="T4" s="2" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="U4" s="2" t="s">
         <v>31</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="W4" s="2" t="s">
         <v>31</v>
       </c>
       <c r="X4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z4" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="24" t="s">
+        <v>242</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C5" s="3">
+      <c r="E5" s="3">
         <v>46327</v>
       </c>
-      <c r="D5" s="3">
+      <c r="F5" s="3">
         <v>46346</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="G5" s="2">
-        <v>2</v>
-      </c>
-      <c r="H5" s="2">
-        <v>2</v>
       </c>
       <c r="I5" s="2">
         <v>2</v>
       </c>
       <c r="J5" s="2">
+        <v>2</v>
+      </c>
+      <c r="K5" s="2">
+        <v>2</v>
+      </c>
+      <c r="L5" s="2">
         <v>1</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="M5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="N5" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="O5" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="P5" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="O5" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="P5" s="2" t="s">
+      <c r="Q5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="R5" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="Q5" s="4" t="s">
+      <c r="S5" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="S5" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="T5" s="2" t="s">
         <v>31</v>
       </c>
@@ -2446,78 +2602,84 @@
         <v>31</v>
       </c>
       <c r="V5" s="2" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="W5" s="2" t="s">
         <v>31</v>
       </c>
       <c r="X5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z5" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="24" t="s">
+        <v>242</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="5">
+      <c r="E6" s="5">
         <v>46327</v>
       </c>
-      <c r="D6" s="3">
+      <c r="F6" s="3">
         <v>46346</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="G6" s="2">
+      <c r="I6" s="2">
         <v>4</v>
       </c>
-      <c r="H6" s="2">
+      <c r="J6" s="2">
         <v>2</v>
       </c>
-      <c r="I6" s="2">
+      <c r="K6" s="2">
         <v>2</v>
       </c>
-      <c r="J6" s="2">
+      <c r="L6" s="2">
         <v>1</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="M6" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="N6" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="M6" s="2" t="s">
+      <c r="O6" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="N6" s="2" t="s">
+      <c r="P6" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="O6" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="P6" s="2" t="s">
+      <c r="Q6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="R6" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="Q6" s="4" t="s">
+      <c r="S6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R6" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S6" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="T6" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="U6" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="V6" s="2" t="s">
         <v>31</v>
@@ -2526,143 +2688,155 @@
         <v>31</v>
       </c>
       <c r="X6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z6" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="24" t="s">
+        <v>242</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C7" s="3">
+      <c r="E7" s="3">
         <v>46327</v>
       </c>
-      <c r="D7" s="3">
+      <c r="F7" s="3">
         <v>46346</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="G7" s="2">
-        <v>1</v>
-      </c>
-      <c r="H7" s="2">
-        <v>2</v>
       </c>
       <c r="I7" s="2">
         <v>1</v>
       </c>
       <c r="J7" s="2">
+        <v>2</v>
+      </c>
+      <c r="K7" s="2">
+        <v>1</v>
+      </c>
+      <c r="L7" s="2">
         <v>0</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="M7" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="N7" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="O7" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="P7" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="O7" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="P7" s="2" t="s">
+      <c r="Q7" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="R7" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="Q7" s="4" t="s">
+      <c r="S7" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R7" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S7" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="T7" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="U7" s="2" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="V7" s="2" t="s">
         <v>31</v>
       </c>
       <c r="W7" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="X7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z7" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C8" s="5">
+      <c r="E8" s="5">
         <v>46327</v>
       </c>
-      <c r="D8" s="3">
+      <c r="F8" s="3">
         <v>46346</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="G8" s="2">
+      <c r="I8" s="2">
         <v>2</v>
-      </c>
-      <c r="H8" s="2">
-        <v>1</v>
-      </c>
-      <c r="I8" s="2">
-        <v>1</v>
       </c>
       <c r="J8" s="2">
         <v>1</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="K8" s="2">
+        <v>1</v>
+      </c>
+      <c r="L8" s="2">
+        <v>1</v>
+      </c>
+      <c r="M8" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="N8" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="O8" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="N8" s="2" t="s">
+      <c r="P8" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="O8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="P8" s="2" t="s">
+      <c r="Q8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="R8" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="Q8" s="4" t="s">
+      <c r="S8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S8" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="T8" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="U8" s="2" t="s">
         <v>31</v>
@@ -2671,70 +2845,76 @@
         <v>31</v>
       </c>
       <c r="W8" s="2" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="X8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z8" s="2" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="3">
+      <c r="E9" s="3">
         <v>46327</v>
       </c>
-      <c r="D9" s="3">
+      <c r="F9" s="3">
         <v>46346</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="G9" s="2">
+      <c r="I9" s="2">
         <v>3</v>
       </c>
-      <c r="H9" s="2">
+      <c r="J9" s="2">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="K9" s="2">
         <v>2</v>
       </c>
-      <c r="J9" s="2">
+      <c r="L9" s="2">
         <v>1</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="M9" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="N9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="M9" s="2" t="s">
+      <c r="O9" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="N9" s="2" t="s">
+      <c r="P9" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="O9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P9" s="2" t="s">
+      <c r="Q9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R9" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="Q9" s="4" t="s">
+      <c r="S9" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="S9" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="T9" s="2" t="s">
         <v>31</v>
       </c>
@@ -2745,144 +2925,156 @@
         <v>31</v>
       </c>
       <c r="W9" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="X9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z9" s="2" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="5">
+      <c r="E10" s="5">
         <v>46327</v>
       </c>
-      <c r="D10" s="3">
+      <c r="F10" s="3">
         <v>46346</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="G10" s="2">
+      <c r="I10" s="2">
         <v>1</v>
       </c>
-      <c r="H10" s="2">
+      <c r="J10" s="2">
         <v>4</v>
       </c>
-      <c r="I10" s="2">
+      <c r="K10" s="2">
         <v>2</v>
       </c>
-      <c r="J10" s="2">
+      <c r="L10" s="2">
         <v>2</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="M10" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="N10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="M10" s="2" t="s">
+      <c r="O10" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="N10" s="2" t="s">
+      <c r="P10" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="O10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P10" s="2" t="s">
+      <c r="Q10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R10" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="Q10" s="4" t="s">
+      <c r="S10" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="S10" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="T10" s="2" t="s">
         <v>31</v>
       </c>
       <c r="U10" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="V10" s="2" t="s">
         <v>31</v>
       </c>
       <c r="W10" s="2" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="X10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z10" s="2" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C11" s="3">
+      <c r="E11" s="3">
         <v>46327</v>
       </c>
-      <c r="D11" s="3">
+      <c r="F11" s="3">
         <v>46346</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G11" s="2">
+      <c r="I11" s="2">
         <v>9</v>
-      </c>
-      <c r="H11" s="2">
-        <v>0</v>
-      </c>
-      <c r="I11" s="2">
-        <v>0</v>
       </c>
       <c r="J11" s="2">
         <v>0</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="K11" s="2">
+        <v>0</v>
+      </c>
+      <c r="L11" s="2">
+        <v>0</v>
+      </c>
+      <c r="M11" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="L11" s="2" t="s">
+      <c r="N11" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="M11" s="2" t="s">
+      <c r="O11" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="N11" s="2" t="s">
+      <c r="P11" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="O11" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P11" s="2" t="s">
+      <c r="Q11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R11" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="Q11" s="4" t="s">
+      <c r="S11" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R11" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="S11" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="T11" s="2" t="s">
         <v>31</v>
       </c>
@@ -2896,203 +3088,218 @@
         <v>31</v>
       </c>
       <c r="X11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z11" s="2" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>197</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="5">
+      <c r="E12" s="5">
         <v>46327</v>
       </c>
-      <c r="D12" s="3">
+      <c r="F12" s="3">
         <v>46346</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="G12" s="2">
+      <c r="I12" s="2">
         <v>1</v>
       </c>
-      <c r="H12" s="2">
+      <c r="J12" s="2">
         <v>2</v>
       </c>
-      <c r="I12" s="2">
+      <c r="K12" s="2">
         <v>3</v>
       </c>
-      <c r="J12" s="2">
+      <c r="L12" s="2">
         <v>3</v>
       </c>
-      <c r="K12" s="2" t="s">
+      <c r="M12" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="L12" s="2" t="s">
+      <c r="N12" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="M12" s="2" t="s">
+      <c r="O12" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="N12" s="2" t="s">
+      <c r="P12" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="O12" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P12" s="2" t="s">
+      <c r="Q12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R12" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="Q12" s="4" t="s">
+      <c r="S12" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R12" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="S12" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="T12" s="2" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="U12" s="2" t="s">
         <v>42</v>
       </c>
       <c r="V12" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="W12" s="2" t="s">
         <v>42</v>
       </c>
       <c r="X12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y12" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z12" s="2" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:26" s="23" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>241</v>
+      </c>
+      <c r="D13" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" s="20">
+        <v>46327</v>
+      </c>
+      <c r="F13" s="21">
+        <v>46346</v>
+      </c>
+      <c r="G13" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H13" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="I13" s="19">
+        <v>3</v>
+      </c>
+      <c r="J13" s="19">
+        <v>3</v>
+      </c>
+      <c r="K13" s="19">
+        <v>3</v>
+      </c>
+      <c r="L13" s="19">
+        <v>3</v>
+      </c>
+      <c r="M13" s="19" t="s">
+        <v>200</v>
+      </c>
+      <c r="N13" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="O13" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="P13" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="5">
-        <v>46327</v>
-      </c>
-      <c r="D13" s="3">
-        <v>46346</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="G13" s="2">
-        <v>3</v>
-      </c>
-      <c r="H13" s="2">
-        <v>3</v>
-      </c>
-      <c r="I13" s="2">
-        <v>3</v>
-      </c>
-      <c r="J13" s="2">
-        <v>3</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="O13" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="P13" s="2" t="s">
+      <c r="Q13" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="R13" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="Q13" s="4" t="s">
+      <c r="S13" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="R13" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S13" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="T13" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="U13" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="V13" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="W13" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="X13" s="2" t="s">
+      <c r="T13" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="U13" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="V13" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="W13" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="X13" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y13" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z13" s="19" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="6"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="7"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
       <c r="D20" s="8"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="9"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="9"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="7"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
       <c r="D23" s="8"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="9"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="12"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
       <c r="D25" s="12"/>
       <c r="E25" s="12"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="10"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A25:E25"/>
-  </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="Q2" r:id="rId1" xr:uid="{9EBB1B09-03B2-4B26-A3F0-C9A7560603A1}"/>
-    <hyperlink ref="Q3:Q12" r:id="rId2" display="accept@accept.com" xr:uid="{2E690355-2D2B-44AC-B2CA-4DDFE3882727}"/>
-    <hyperlink ref="Q13" r:id="rId3" xr:uid="{DA7FA2D3-6C56-483A-8DB3-CE9612529E40}"/>
+    <hyperlink ref="S2" r:id="rId1" xr:uid="{9EBB1B09-03B2-4B26-A3F0-C9A7560603A1}"/>
+    <hyperlink ref="S3:S12" r:id="rId2" display="accept@accept.com" xr:uid="{2E690355-2D2B-44AC-B2CA-4DDFE3882727}"/>
+    <hyperlink ref="S13" r:id="rId3" xr:uid="{DA7FA2D3-6C56-483A-8DB3-CE9612529E40}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mejor manejo de bundle
</commit_message>
<xml_diff>
--- a/data/maestro.xlsx
+++ b/data/maestro.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://everisgroup-my.sharepoint.com/personal/dnarvaec_emeal_nttdata_com1/Documents/Documents/Proyectos AUTO/Avianca/Automatizacion/auto_avianca/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dnarvaec\OneDrive - NTT DATA EMEAL\Documents\Proyectos AUTO\Avianca\Automatizacion\auto_avianca\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="73" documentId="8_{48F3D4DC-C1BA-440D-80D9-C9B78812467E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96EB83F1-F7E9-4C2C-BC7E-032FCFA188C2}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DCD6B92-4D75-475E-87BE-573573B3FABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NBF_OW" sheetId="5" r:id="rId1"/>
@@ -922,7 +922,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -984,6 +984,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1614,83 +1618,83 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:26" s="23" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="19" t="s">
         <v>180</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="19" t="s">
         <v>242</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="19" t="s">
         <v>235</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="21">
         <v>46327</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="19">
         <v>3</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="19">
         <v>2</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="19">
         <v>2</v>
       </c>
-      <c r="L5" s="2">
+      <c r="L5" s="19">
         <v>2</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="M5" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="N5" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="O5" s="2" t="s">
+      <c r="O5" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="P5" s="2" t="s">
+      <c r="P5" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="Q5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="R5" s="2" t="s">
+      <c r="Q5" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="R5" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="S5" s="4" t="s">
+      <c r="S5" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="T5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="U5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="V5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="W5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="X5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="Y5" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="Z5" s="2" t="s">
+      <c r="T5" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="U5" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="V5" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="W5" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="X5" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y5" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z5" s="19" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1774,83 +1778,83 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:26" s="23" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="19" t="s">
         <v>182</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="19" t="s">
         <v>231</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="19" t="s">
         <v>237</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="21">
         <v>46327</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="19">
         <v>2</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="19">
         <v>0</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="19">
         <v>1</v>
       </c>
-      <c r="L7" s="2">
+      <c r="L7" s="19">
         <v>1</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="M7" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="N7" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="O7" s="2" t="s">
+      <c r="O7" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="P7" s="2" t="s">
+      <c r="P7" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="Q7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="R7" s="2" t="s">
+      <c r="Q7" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="R7" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="S7" s="4" t="s">
+      <c r="S7" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="T7" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="U7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="V7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="W7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="X7" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="Z7" s="2" t="s">
+      <c r="T7" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="U7" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="V7" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="W7" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="X7" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y7" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z7" s="19" t="s">
         <v>88</v>
       </c>
     </row>
@@ -2014,83 +2018,83 @@
         <v>104</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:26" s="26" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="24" t="s">
         <v>185</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="24" t="s">
         <v>231</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="24" t="s">
         <v>240</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="25">
         <v>46327</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="24">
         <v>2</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="24">
         <v>2</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="24">
         <v>2</v>
       </c>
-      <c r="L10" s="2">
+      <c r="L10" s="24">
         <v>2</v>
       </c>
-      <c r="M10" s="2" t="s">
+      <c r="M10" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="N10" s="2" t="s">
+      <c r="N10" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="O10" s="2" t="s">
+      <c r="O10" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="P10" s="2" t="s">
+      <c r="P10" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="Q10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="R10" s="2" t="s">
+      <c r="Q10" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="R10" s="24" t="s">
         <v>111</v>
       </c>
       <c r="S10" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="T10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="U10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="V10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="W10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="X10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="Z10" s="2" t="s">
+      <c r="T10" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="U10" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="V10" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="W10" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="X10" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y10" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z10" s="24" t="s">
         <v>112</v>
       </c>
     </row>
@@ -2385,7 +2389,7 @@
         <v>242</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="D3" s="19" t="s">
         <v>38</v>
@@ -2541,7 +2545,7 @@
       <c r="A5" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="2" t="s">
         <v>242</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -2621,7 +2625,7 @@
       <c r="A6" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="2" t="s">
         <v>242</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -2701,7 +2705,7 @@
       <c r="A7" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="2" t="s">
         <v>242</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -2781,7 +2785,7 @@
       <c r="A8" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="2" t="s">
         <v>231</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -2861,7 +2865,7 @@
       <c r="A9" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="2" t="s">
         <v>231</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -2941,7 +2945,7 @@
       <c r="A10" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="2" t="s">
         <v>231</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -3021,7 +3025,7 @@
       <c r="A11" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="2" t="s">
         <v>231</v>
       </c>
       <c r="C11" s="2" t="s">

</xml_diff>

<commit_message>
EJEMPLO Promotion pagew finalizado y testeado
</commit_message>
<xml_diff>
--- a/data/maestro.xlsx
+++ b/data/maestro.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dnarvaec\OneDrive - NTT DATA EMEAL\Documents\Proyectos AUTO\Avianca\Automatizacion\auto_avianca\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://everisgroup-my.sharepoint.com/personal/dnarvaec_emeal_nttdata_com1/Documents/Documents/Proyectos AUTO/Avianca/Automatizacion/auto_avianca/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1137B3C4-6E13-4691-8E16-D9EA49B97E1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{1137B3C4-6E13-4691-8E16-D9EA49B97E1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{151AEA2A-5702-45D5-8BDA-5331CDAB0B96}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NBF_OW" sheetId="5" r:id="rId1"/>
@@ -922,7 +922,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -981,6 +981,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1771,83 +1778,83 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:26" s="23" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="19" t="s">
+    <row r="7" spans="1:26" s="26" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="24" t="s">
         <v>231</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="24" t="s">
         <v>237</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" s="25">
+        <v>46327</v>
+      </c>
+      <c r="F7" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="H7" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="I7" s="24">
+        <v>2</v>
+      </c>
+      <c r="J7" s="24">
+        <v>0</v>
+      </c>
+      <c r="K7" s="24">
+        <v>1</v>
+      </c>
+      <c r="L7" s="24">
+        <v>1</v>
+      </c>
+      <c r="M7" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="N7" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="O7" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="P7" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="21">
-        <v>46327</v>
-      </c>
-      <c r="F7" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="G7" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="H7" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="I7" s="19">
-        <v>2</v>
-      </c>
-      <c r="J7" s="19">
-        <v>0</v>
-      </c>
-      <c r="K7" s="19">
-        <v>1</v>
-      </c>
-      <c r="L7" s="19">
-        <v>1</v>
-      </c>
-      <c r="M7" s="19" t="s">
-        <v>85</v>
-      </c>
-      <c r="N7" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="O7" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="P7" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q7" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="R7" s="19" t="s">
+      <c r="Q7" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="R7" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="S7" s="22" t="s">
+      <c r="S7" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="T7" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="U7" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="V7" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="W7" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="X7" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y7" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="Z7" s="19" t="s">
+      <c r="T7" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="U7" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="V7" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="W7" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="X7" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y7" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z7" s="24" t="s">
         <v>88</v>
       </c>
     </row>
@@ -2374,83 +2381,83 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:26" s="23" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="19" t="s">
+    <row r="3" spans="1:26" s="26" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="24" t="s">
         <v>188</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="24" t="s">
         <v>242</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="24" t="s">
         <v>237</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="E3" s="21">
+      <c r="E3" s="25">
         <v>46327</v>
       </c>
-      <c r="F3" s="21">
+      <c r="F3" s="25">
         <v>46346</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="I3" s="19">
+      <c r="I3" s="24">
         <v>1</v>
       </c>
-      <c r="J3" s="19">
+      <c r="J3" s="24">
         <v>1</v>
       </c>
-      <c r="K3" s="19">
+      <c r="K3" s="24">
         <v>0</v>
       </c>
-      <c r="L3" s="19">
+      <c r="L3" s="24">
         <v>0</v>
       </c>
-      <c r="M3" s="19" t="s">
+      <c r="M3" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="N3" s="19" t="s">
+      <c r="N3" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="O3" s="19" t="s">
+      <c r="O3" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="P3" s="19" t="s">
+      <c r="P3" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="Q3" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="R3" s="19" t="s">
+      <c r="Q3" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="R3" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="S3" s="22" t="s">
+      <c r="S3" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="T3" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="U3" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="V3" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="W3" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="X3" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="Y3" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="Z3" s="19" t="s">
+      <c r="T3" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="U3" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="V3" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="W3" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="X3" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y3" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z3" s="24" t="s">
         <v>44</v>
       </c>
     </row>

</xml_diff>